<commit_message>
Added new RDF data schemes and visual schemes, and fixed xlsx-spreadsheets for economy-table30-34
</commit_message>
<xml_diff>
--- a/sources/table_normalization/xlsx/economy-table30.xlsx
+++ b/sources/table_normalization/xlsx/economy-table30.xlsx
@@ -404,7 +404,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -413,6 +413,7 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -786,7 +787,7 @@
       </c>
     </row>
     <row r="2" spans="1:11">
-      <c r="A2" s="5"/>
+      <c r="A2" s="8"/>
       <c r="B2" s="5" t="s">
         <v>5</v>
       </c>
@@ -800,17 +801,17 @@
       <c r="K2" s="3"/>
     </row>
     <row r="3" spans="1:11">
-      <c r="A3" s="5"/>
-      <c r="B3" s="5" t="s">
+      <c r="A3" s="8"/>
+      <c r="B3" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="E3" s="5"/>
+      <c r="E3" s="8"/>
       <c r="G3" s="2"/>
       <c r="H3" s="3"/>
       <c r="I3" s="3"/>
@@ -818,7 +819,7 @@
       <c r="K3" s="3"/>
     </row>
     <row r="4" spans="1:11">
-      <c r="A4" s="5"/>
+      <c r="A4" s="8"/>
       <c r="B4" s="5" t="s">
         <v>9</v>
       </c>

</xml_diff>